<commit_message>
added model.py showing empirical model and data points
</commit_message>
<xml_diff>
--- a/data/2026-06-16_15-50-10_OpeningAngleVariation/analysis.xlsx
+++ b/data/2026-06-16_15-50-10_OpeningAngleVariation/analysis.xlsx
@@ -1,24 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tmdacjp-my.sharepoint.com/personal/koch_f_f64c_m_isct_ac_jp/Documents/Documents/4-Software/data/2026-06-16_15-50-10_OpeningAngleVariation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{66EBF3FB-79E4-4729-AD1B-470CE93A4271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6688B195-280A-4EC8-9E51-D5481E3C0352}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{66EBF3FB-79E4-4729-AD1B-470CE93A4271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B6FE3B8-0805-4142-A7F4-7C69F5B3B7D7}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F4D94018-A683-4337-8E84-0B45674183A7}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{F4D94018-A683-4337-8E84-0B45674183A7}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1232,7 +1240,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1447,8 +1455,18 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="el-GR"/>
-                  <a:t>α</a:t>
+                  <a:rPr lang="en-GB" baseline="0">
+                    <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                    <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  </a:rPr>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="el-GR" baseline="0">
+                    <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                    <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  </a:rPr>
+                  <a:t>θ</a:t>
                 </a:r>
                 <a:r>
                   <a:rPr lang="en-GB" baseline="0"/>
@@ -1608,7 +1626,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1663,6 +1681,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1670,7 +1689,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3223,13 +3241,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8BFBD16-B9C5-43E7-BB91-6B1E1D40C980}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3237,7 +3255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -3245,7 +3263,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -3253,7 +3271,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -3261,12 +3279,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3274,7 +3292,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -3282,7 +3300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -3308,7 +3326,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>1</v>
       </c>
@@ -3335,7 +3353,7 @@
         <v>-0.10515905481978501</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>2</v>
       </c>
@@ -3362,7 +3380,7 @@
         <v>1.12729562380548E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>3</v>
       </c>
@@ -3389,7 +3407,7 @@
         <v>9.6885166655364899E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>4</v>
       </c>
@@ -3416,7 +3434,7 @@
         <v>2.64171747876593E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>5</v>
       </c>
@@ -3443,7 +3461,7 @@
         <v>-3.5498213328473999E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>6</v>
       </c>
@@ -3470,7 +3488,7 @@
         <v>-5.7623253334126599E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>7</v>
       </c>
@@ -3497,7 +3515,7 @@
         <v>0.216996047779806</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>8</v>
       </c>
@@ -3524,7 +3542,7 @@
         <v>-3.3039481016707999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>9</v>
       </c>
@@ -3551,7 +3569,7 @@
         <v>3.1434363672842199E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>10</v>
       </c>
@@ -3578,7 +3596,7 @@
         <v>-1.6831351814634701E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>11</v>
       </c>
@@ -3605,7 +3623,7 @@
         <v>-5.2946746879927301E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>12</v>
       </c>
@@ -3632,7 +3650,7 @@
         <v>6.64429979698304E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>13</v>
       </c>

</xml_diff>